<commit_message>
Latest workshop methods and figures
</commit_message>
<xml_diff>
--- a/Indicator_4/Blank_data/EcoTest_Input.xlsx
+++ b/Indicator_4/Blank_data/EcoTest_Input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\EcoTest_Train\Indicator_4\Real_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\EcoTest_Train\Indicator_4\Blank_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CFEE16-C983-4CAC-9BEC-C6F48784A27B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87F6703-02FD-4A2E-9040-E1E682A22F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="1" xr2:uid="{F62724AB-7BA1-4BCA-888B-66476DD5ABBE}"/>
   </bookViews>
@@ -736,9 +736,7 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6">
-        <v>15.22</v>
-      </c>
+      <c r="B3" s="6"/>
       <c r="C3" t="s">
         <v>5</v>
       </c>
@@ -753,9 +751,7 @@
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6">
-        <v>0.21</v>
-      </c>
+      <c r="B4" s="6"/>
       <c r="C4" t="s">
         <v>4</v>
       </c>
@@ -770,9 +766,7 @@
       <c r="A5" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="6">
-        <v>122.34</v>
-      </c>
+      <c r="B5" s="6"/>
       <c r="C5" t="s">
         <v>68</v>
       </c>
@@ -787,9 +781,7 @@
       <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="5">
-        <v>0.65</v>
-      </c>
+      <c r="B6" s="5"/>
       <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
@@ -804,9 +796,7 @@
       <c r="A7" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="6">
-        <v>0.49</v>
-      </c>
+      <c r="B7" s="6"/>
       <c r="C7" t="s">
         <v>36</v>
       </c>
@@ -821,9 +811,7 @@
       <c r="A8" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="6">
-        <v>1.05</v>
-      </c>
+      <c r="B8" s="6"/>
       <c r="C8" t="s">
         <v>37</v>
       </c>
@@ -838,9 +826,7 @@
       <c r="A9" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="5">
-        <v>0.97</v>
-      </c>
+      <c r="B9" s="5"/>
       <c r="C9" s="4" t="s">
         <v>38</v>
       </c>
@@ -855,9 +841,7 @@
       <c r="A10" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="6">
-        <v>0.35</v>
-      </c>
+      <c r="B10" s="6"/>
       <c r="C10" t="s">
         <v>36</v>
       </c>
@@ -872,9 +856,7 @@
       <c r="A11" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="6">
-        <v>1.05</v>
-      </c>
+      <c r="B11" s="6"/>
       <c r="C11" t="s">
         <v>37</v>
       </c>
@@ -889,9 +871,7 @@
       <c r="A12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="5">
-        <v>0.97</v>
-      </c>
+      <c r="B12" s="5"/>
       <c r="C12" s="4" t="s">
         <v>38</v>
       </c>
@@ -906,9 +886,7 @@
       <c r="A13" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="6">
-        <v>0.32</v>
-      </c>
+      <c r="B13" s="6"/>
       <c r="C13" t="s">
         <v>36</v>
       </c>
@@ -923,9 +901,7 @@
       <c r="A14" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="6">
-        <v>0.95</v>
-      </c>
+      <c r="B14" s="6"/>
       <c r="C14" t="s">
         <v>37</v>
       </c>
@@ -940,9 +916,7 @@
       <c r="A15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="5">
-        <v>0.99</v>
-      </c>
+      <c r="B15" s="5"/>
       <c r="C15" s="4" t="s">
         <v>38</v>
       </c>
@@ -957,9 +931,7 @@
       <c r="A16" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="6">
-        <v>0.45</v>
-      </c>
+      <c r="B16" s="6"/>
       <c r="C16" t="s">
         <v>36</v>
       </c>
@@ -974,9 +946,7 @@
       <c r="A17" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="6">
-        <v>1.36</v>
-      </c>
+      <c r="B17" s="6"/>
       <c r="C17" t="s">
         <v>37</v>
       </c>
@@ -991,9 +961,7 @@
       <c r="A18" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="5">
-        <v>0.88</v>
-      </c>
+      <c r="B18" s="5"/>
       <c r="C18" s="4" t="s">
         <v>38</v>
       </c>
@@ -1008,9 +976,7 @@
       <c r="A19" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="6">
-        <v>0.41</v>
-      </c>
+      <c r="B19" s="6"/>
       <c r="C19" t="s">
         <v>30</v>
       </c>
@@ -1025,9 +991,7 @@
       <c r="A20" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="6">
-        <v>0.39</v>
-      </c>
+      <c r="B20" s="6"/>
       <c r="C20" t="s">
         <v>33</v>
       </c>
@@ -1042,9 +1006,7 @@
       <c r="A21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="5">
-        <v>0.21</v>
-      </c>
+      <c r="B21" s="5"/>
       <c r="C21" s="4" t="s">
         <v>34</v>
       </c>
@@ -1163,19 +1125,12 @@
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="1">
-        <v>1950</v>
-      </c>
-      <c r="B2" s="9">
-        <v>131.691</v>
-      </c>
+      <c r="B2" s="9"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
-      <c r="G2" s="10">
-        <v>1.2210000000000001</v>
-      </c>
+      <c r="G2" s="10"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
@@ -1196,19 +1151,12 @@
       <c r="Y2" s="8"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="1">
-        <v>1951</v>
-      </c>
-      <c r="B3" s="9">
-        <v>754.221</v>
-      </c>
+      <c r="B3" s="9"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="10">
-        <v>1.22</v>
-      </c>
+      <c r="G3" s="10"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
@@ -1229,19 +1177,12 @@
       <c r="Y3" s="8"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="1">
-        <v>1952</v>
-      </c>
-      <c r="B4" s="9">
-        <v>1707.8330000000001</v>
-      </c>
+      <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
-      <c r="G4" s="10">
-        <v>1.22</v>
-      </c>
+      <c r="G4" s="10"/>
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
@@ -1262,19 +1203,12 @@
       <c r="Y4" s="8"/>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="1">
-        <v>1953</v>
-      </c>
-      <c r="B5" s="9">
-        <v>1973.704</v>
-      </c>
+      <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
-      <c r="G5" s="10">
-        <v>1.22</v>
-      </c>
+      <c r="G5" s="10"/>
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
       <c r="J5" s="7"/>
@@ -1295,19 +1229,12 @@
       <c r="Y5" s="8"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="1">
-        <v>1954</v>
-      </c>
-      <c r="B6" s="9">
-        <v>3933.6790000000001</v>
-      </c>
+      <c r="B6" s="9"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
-      <c r="G6" s="10">
-        <v>1.22</v>
-      </c>
+      <c r="G6" s="10"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
@@ -1328,19 +1255,12 @@
       <c r="Y6" s="8"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="1">
-        <v>1955</v>
-      </c>
-      <c r="B7" s="9">
-        <v>4394.2849999999999</v>
-      </c>
+      <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
-      <c r="G7" s="10">
-        <v>1.216</v>
-      </c>
+      <c r="G7" s="10"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
@@ -1361,19 +1281,12 @@
       <c r="Y7" s="8"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="1">
-        <v>1956</v>
-      </c>
-      <c r="B8" s="9">
-        <v>4051.817</v>
-      </c>
+      <c r="B8" s="9"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
-      <c r="G8" s="10">
-        <v>1.2110000000000001</v>
-      </c>
+      <c r="G8" s="10"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
@@ -1394,19 +1307,12 @@
       <c r="Y8" s="8"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="1">
-        <v>1957</v>
-      </c>
-      <c r="B9" s="9">
-        <v>4951.7619999999997</v>
-      </c>
+      <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
-      <c r="G9" s="10">
-        <v>1.1990000000000001</v>
-      </c>
+      <c r="G9" s="10"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
@@ -1427,19 +1333,12 @@
       <c r="Y9" s="8"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="1">
-        <v>1958</v>
-      </c>
-      <c r="B10" s="9">
-        <v>4791.3789999999999</v>
-      </c>
+      <c r="B10" s="9"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
-      <c r="G10" s="10">
-        <v>1.1850000000000001</v>
-      </c>
+      <c r="G10" s="10"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
@@ -1460,19 +1359,12 @@
       <c r="Y10" s="8"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="1">
-        <v>1959</v>
-      </c>
-      <c r="B11" s="9">
-        <v>5024.2539999999999</v>
-      </c>
+      <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
-      <c r="G11" s="10">
-        <v>1.173</v>
-      </c>
+      <c r="G11" s="10"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
@@ -1493,19 +1385,12 @@
       <c r="Y11" s="8"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="1">
-        <v>1960</v>
-      </c>
-      <c r="B12" s="9">
-        <v>4587.0129999999999</v>
-      </c>
+      <c r="B12" s="9"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
-      <c r="G12" s="10">
-        <v>1.1579999999999999</v>
-      </c>
+      <c r="G12" s="10"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
@@ -1526,19 +1411,12 @@
       <c r="Y12" s="8"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="1">
-        <v>1961</v>
-      </c>
-      <c r="B13" s="9">
-        <v>4508.3549999999996</v>
-      </c>
+      <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
-      <c r="G13" s="10">
-        <v>1.145</v>
-      </c>
+      <c r="G13" s="10"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
       <c r="J13" s="7"/>
@@ -1559,19 +1437,12 @@
       <c r="Y13" s="8"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="1">
-        <v>1962</v>
-      </c>
-      <c r="B14" s="9">
-        <v>4944.6790000000001</v>
-      </c>
+      <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
-      <c r="G14" s="10">
-        <v>1.133</v>
-      </c>
+      <c r="G14" s="10"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
@@ -1592,19 +1463,12 @@
       <c r="Y14" s="8"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="1">
-        <v>1963</v>
-      </c>
-      <c r="B15" s="9">
-        <v>5859.4170000000004</v>
-      </c>
+      <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
-      <c r="G15" s="10">
-        <v>1.1220000000000001</v>
-      </c>
+      <c r="G15" s="10"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="7"/>
@@ -1625,19 +1489,12 @@
       <c r="Y15" s="8"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="1">
-        <v>1964</v>
-      </c>
-      <c r="B16" s="9">
-        <v>6521.1850000000004</v>
-      </c>
+      <c r="B16" s="9"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="10">
-        <v>1.115</v>
-      </c>
+      <c r="G16" s="10"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
@@ -1657,20 +1514,13 @@
       <c r="X16" s="7"/>
       <c r="Y16" s="8"/>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="1">
-        <v>1965</v>
-      </c>
-      <c r="B17" s="9">
-        <v>4479.4859999999999</v>
-      </c>
+    <row r="17" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B17" s="9"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
-      <c r="G17" s="10">
-        <v>1.107</v>
-      </c>
+      <c r="G17" s="10"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
@@ -1690,20 +1540,13 @@
       <c r="X17" s="7"/>
       <c r="Y17" s="8"/>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="1">
-        <v>1966</v>
-      </c>
-      <c r="B18" s="9">
-        <v>5472.7790000000005</v>
-      </c>
+    <row r="18" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18" s="9"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
-      <c r="G18" s="10">
-        <v>1.097</v>
-      </c>
+      <c r="G18" s="10"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
       <c r="J18" s="7"/>
@@ -1723,20 +1566,13 @@
       <c r="X18" s="7"/>
       <c r="Y18" s="8"/>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="1">
-        <v>1967</v>
-      </c>
-      <c r="B19" s="9">
-        <v>8939.8160000000007</v>
-      </c>
+    <row r="19" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" s="9"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
-      <c r="G19" s="10">
-        <v>1.085</v>
-      </c>
+      <c r="G19" s="10"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
       <c r="J19" s="7"/>
@@ -1756,20 +1592,13 @@
       <c r="X19" s="7"/>
       <c r="Y19" s="8"/>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="1">
-        <v>1968</v>
-      </c>
-      <c r="B20" s="9">
-        <v>8621.1470000000008</v>
-      </c>
+    <row r="20" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="9"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
-      <c r="G20" s="10">
-        <v>1.0780000000000001</v>
-      </c>
+      <c r="G20" s="10"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
       <c r="J20" s="7"/>
@@ -1789,20 +1618,13 @@
       <c r="X20" s="7"/>
       <c r="Y20" s="8"/>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="1">
-        <v>1969</v>
-      </c>
-      <c r="B21" s="9">
-        <v>9030.3420000000006</v>
-      </c>
+    <row r="21" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B21" s="9"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
-      <c r="G21" s="10">
-        <v>1.071</v>
-      </c>
+      <c r="G21" s="10"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
       <c r="J21" s="7"/>
@@ -1822,20 +1644,13 @@
       <c r="X21" s="7"/>
       <c r="Y21" s="8"/>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="1">
-        <v>1970</v>
-      </c>
-      <c r="B22" s="9">
-        <v>4842.0590000000002</v>
-      </c>
+    <row r="22" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22" s="9"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
-      <c r="G22" s="10">
-        <v>1.0569999999999999</v>
-      </c>
+      <c r="G22" s="10"/>
       <c r="H22" s="7"/>
       <c r="I22" s="7"/>
       <c r="J22" s="7"/>
@@ -1855,20 +1670,13 @@
       <c r="X22" s="7"/>
       <c r="Y22" s="8"/>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="1">
-        <v>1971</v>
-      </c>
-      <c r="B23" s="9">
-        <v>5165.5290000000005</v>
-      </c>
+    <row r="23" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
-      <c r="G23" s="10">
-        <v>1.046</v>
-      </c>
+      <c r="G23" s="10"/>
       <c r="H23" s="7"/>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
@@ -1888,20 +1696,13 @@
       <c r="X23" s="7"/>
       <c r="Y23" s="8"/>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="1">
-        <v>1972</v>
-      </c>
-      <c r="B24" s="9">
-        <v>5123.607</v>
-      </c>
+    <row r="24" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B24" s="9"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
-      <c r="G24" s="10">
-        <v>1.034</v>
-      </c>
+      <c r="G24" s="10"/>
       <c r="H24" s="7"/>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
@@ -1921,20 +1722,13 @@
       <c r="X24" s="7"/>
       <c r="Y24" s="8"/>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="1">
-        <v>1973</v>
-      </c>
-      <c r="B25" s="9">
-        <v>3385.0639999999999</v>
-      </c>
+    <row r="25" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B25" s="9"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
-      <c r="G25" s="10">
-        <v>1.032</v>
-      </c>
+      <c r="G25" s="10"/>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
@@ -1954,20 +1748,13 @@
       <c r="X25" s="7"/>
       <c r="Y25" s="8"/>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="1">
-        <v>1974</v>
-      </c>
-      <c r="B26" s="9">
-        <v>5004.5540000000001</v>
-      </c>
+    <row r="26" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26" s="9"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
-      <c r="G26" s="10">
-        <v>1.03</v>
-      </c>
+      <c r="G26" s="10"/>
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
@@ -1987,20 +1774,13 @@
       <c r="X26" s="7"/>
       <c r="Y26" s="8"/>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="1">
-        <v>1975</v>
-      </c>
-      <c r="B27" s="9">
-        <v>5399.7269999999999</v>
-      </c>
+    <row r="27" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B27" s="9"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
-      <c r="G27" s="10">
-        <v>1.0309999999999999</v>
-      </c>
+      <c r="G27" s="10"/>
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
@@ -2020,20 +1800,13 @@
       <c r="X27" s="7"/>
       <c r="Y27" s="8"/>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="1">
-        <v>1976</v>
-      </c>
-      <c r="B28" s="9">
-        <v>4636.0339999999997</v>
-      </c>
+    <row r="28" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B28" s="9"/>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
-      <c r="G28" s="10">
-        <v>1.0369999999999999</v>
-      </c>
+      <c r="G28" s="10"/>
       <c r="H28" s="7"/>
       <c r="I28" s="7"/>
       <c r="J28" s="7"/>
@@ -2053,20 +1826,13 @@
       <c r="X28" s="7"/>
       <c r="Y28" s="8"/>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="1">
-        <v>1977</v>
-      </c>
-      <c r="B29" s="9">
-        <v>5048.116</v>
-      </c>
+    <row r="29" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B29" s="9"/>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
-      <c r="G29" s="10">
-        <v>1.0389999999999999</v>
-      </c>
+      <c r="G29" s="10"/>
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
@@ -2086,20 +1852,13 @@
       <c r="X29" s="7"/>
       <c r="Y29" s="8"/>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="1">
-        <v>1978</v>
-      </c>
-      <c r="B30" s="9">
-        <v>6252.3329999999996</v>
-      </c>
+    <row r="30" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B30" s="9"/>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
-      <c r="G30" s="10">
-        <v>1.042</v>
-      </c>
+      <c r="G30" s="10"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
@@ -2119,20 +1878,13 @@
       <c r="X30" s="7"/>
       <c r="Y30" s="8"/>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="1">
-        <v>1979</v>
-      </c>
-      <c r="B31" s="9">
-        <v>7963.2719999999999</v>
-      </c>
+    <row r="31" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B31" s="9"/>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
-      <c r="G31" s="10">
-        <v>1.0469999999999999</v>
-      </c>
+      <c r="G31" s="10"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
@@ -2152,20 +1904,13 @@
       <c r="X31" s="7"/>
       <c r="Y31" s="8"/>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="1">
-        <v>1980</v>
-      </c>
-      <c r="B32" s="9">
-        <v>7532.7960000000003</v>
-      </c>
+    <row r="32" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B32" s="9"/>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
-      <c r="G32" s="10">
-        <v>1.052</v>
-      </c>
+      <c r="G32" s="10"/>
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
       <c r="J32" s="7"/>
@@ -2185,20 +1930,13 @@
       <c r="X32" s="7"/>
       <c r="Y32" s="8"/>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="1">
-        <v>1981</v>
-      </c>
-      <c r="B33" s="9">
-        <v>10300.058000000001</v>
-      </c>
+    <row r="33" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B33" s="9"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
-      <c r="G33" s="10">
-        <v>1.056</v>
-      </c>
+      <c r="G33" s="10"/>
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
       <c r="J33" s="7"/>
@@ -2218,20 +1956,13 @@
       <c r="X33" s="7"/>
       <c r="Y33" s="8"/>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="1">
-        <v>1982</v>
-      </c>
-      <c r="B34" s="9">
-        <v>9447.5830000000005</v>
-      </c>
+    <row r="34" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B34" s="9"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
-      <c r="G34" s="10">
-        <v>1.056</v>
-      </c>
+      <c r="G34" s="10"/>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="7"/>
@@ -2251,20 +1982,13 @@
       <c r="X34" s="7"/>
       <c r="Y34" s="8"/>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="1">
-        <v>1983</v>
-      </c>
-      <c r="B35" s="9">
-        <v>10959.38</v>
-      </c>
+    <row r="35" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B35" s="9"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
-      <c r="G35" s="10">
-        <v>1.0569999999999999</v>
-      </c>
+      <c r="G35" s="10"/>
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="7"/>
@@ -2284,20 +2008,13 @@
       <c r="X35" s="7"/>
       <c r="Y35" s="8"/>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="1">
-        <v>1984</v>
-      </c>
-      <c r="B36" s="9">
-        <v>11314.789000000001</v>
-      </c>
+    <row r="36" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B36" s="9"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
-      <c r="G36" s="10">
-        <v>1.054</v>
-      </c>
+      <c r="G36" s="10"/>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="7"/>
@@ -2317,20 +2034,13 @@
       <c r="X36" s="7"/>
       <c r="Y36" s="8"/>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="1">
-        <v>1985</v>
-      </c>
-      <c r="B37" s="9">
-        <v>7028.1589999999997</v>
-      </c>
+    <row r="37" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
       <c r="F37" s="9"/>
-      <c r="G37" s="10">
-        <v>1.054</v>
-      </c>
+      <c r="G37" s="10"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
@@ -2350,20 +2060,13 @@
       <c r="X37" s="7"/>
       <c r="Y37" s="8"/>
     </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="1">
-        <v>1986</v>
-      </c>
-      <c r="B38" s="9">
-        <v>9807.1119999999992</v>
-      </c>
+    <row r="38" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B38" s="9"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
-      <c r="G38" s="10">
-        <v>1.052</v>
-      </c>
+      <c r="G38" s="10"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="7"/>
@@ -2383,20 +2086,13 @@
       <c r="X38" s="7"/>
       <c r="Y38" s="8"/>
     </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="1">
-        <v>1987</v>
-      </c>
-      <c r="B39" s="9">
-        <v>9068.11</v>
-      </c>
+    <row r="39" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B39" s="9"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
-      <c r="G39" s="10">
-        <v>1.0489999999999999</v>
-      </c>
+      <c r="G39" s="10"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="7"/>
@@ -2416,20 +2112,13 @@
       <c r="X39" s="7"/>
       <c r="Y39" s="8"/>
     </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="1">
-        <v>1988</v>
-      </c>
-      <c r="B40" s="9">
-        <v>10414.316000000001</v>
-      </c>
+    <row r="40" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B40" s="9"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
-      <c r="G40" s="10">
-        <v>1.0509999999999999</v>
-      </c>
+      <c r="G40" s="10"/>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
       <c r="J40" s="7"/>
@@ -2449,20 +2138,13 @@
       <c r="X40" s="7"/>
       <c r="Y40" s="8"/>
     </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="1">
-        <v>1989</v>
-      </c>
-      <c r="B41" s="9">
-        <v>13167.272000000001</v>
-      </c>
+    <row r="41" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B41" s="9"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
       <c r="F41" s="9"/>
-      <c r="G41" s="10">
-        <v>1.048</v>
-      </c>
+      <c r="G41" s="10"/>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
       <c r="J41" s="7"/>
@@ -2482,20 +2164,13 @@
       <c r="X41" s="7"/>
       <c r="Y41" s="8"/>
     </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="1">
-        <v>1990</v>
-      </c>
-      <c r="B42" s="9">
-        <v>8256.2939999999999</v>
-      </c>
+    <row r="42" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B42" s="9"/>
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
       <c r="F42" s="9"/>
-      <c r="G42" s="10">
-        <v>1.044</v>
-      </c>
+      <c r="G42" s="10"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
       <c r="J42" s="7"/>
@@ -2515,20 +2190,13 @@
       <c r="X42" s="7"/>
       <c r="Y42" s="8"/>
     </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="1">
-        <v>1991</v>
-      </c>
-      <c r="B43" s="9">
-        <v>10487.235000000001</v>
-      </c>
+    <row r="43" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B43" s="9"/>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
-      <c r="G43" s="10">
-        <v>1.0369999999999999</v>
-      </c>
+      <c r="G43" s="10"/>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
       <c r="J43" s="7"/>
@@ -2548,26 +2216,13 @@
       <c r="X43" s="7"/>
       <c r="Y43" s="8"/>
     </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="1">
-        <v>1992</v>
-      </c>
-      <c r="B44" s="9">
-        <v>10729.145</v>
-      </c>
-      <c r="C44" s="9">
-        <v>128.506</v>
-      </c>
+    <row r="44" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
       <c r="D44" s="9"/>
-      <c r="E44" s="9">
-        <v>0.29599999999999999</v>
-      </c>
-      <c r="F44" s="9">
-        <v>0.373</v>
-      </c>
-      <c r="G44" s="10">
-        <v>1.026</v>
-      </c>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="10"/>
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
       <c r="J44" s="7"/>
@@ -2587,26 +2242,13 @@
       <c r="X44" s="7"/>
       <c r="Y44" s="8"/>
     </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="1">
-        <v>1993</v>
-      </c>
-      <c r="B45" s="9">
-        <v>13087.555</v>
-      </c>
-      <c r="C45" s="9">
-        <v>127.28</v>
-      </c>
+    <row r="45" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
       <c r="D45" s="9"/>
-      <c r="E45" s="9">
-        <v>0.35799999999999998</v>
-      </c>
-      <c r="F45" s="9">
-        <v>0.40400000000000003</v>
-      </c>
-      <c r="G45" s="10">
-        <v>1.0169999999999999</v>
-      </c>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="10"/>
       <c r="H45" s="7"/>
       <c r="I45" s="7"/>
       <c r="J45" s="7"/>
@@ -2626,26 +2268,13 @@
       <c r="X45" s="7"/>
       <c r="Y45" s="8"/>
     </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="1">
-        <v>1994</v>
-      </c>
-      <c r="B46" s="9">
-        <v>17067.864000000001</v>
-      </c>
-      <c r="C46" s="9">
-        <v>121.733</v>
-      </c>
+    <row r="46" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
       <c r="D46" s="9"/>
-      <c r="E46" s="9">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="F46" s="9">
-        <v>0.29699999999999999</v>
-      </c>
-      <c r="G46" s="10">
-        <v>1.0029999999999999</v>
-      </c>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="10"/>
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
       <c r="J46" s="7"/>
@@ -2665,26 +2294,13 @@
       <c r="X46" s="7"/>
       <c r="Y46" s="8"/>
     </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="1">
-        <v>1995</v>
-      </c>
-      <c r="B47" s="9">
-        <v>17570.996999999999</v>
-      </c>
-      <c r="C47" s="9">
-        <v>138.86500000000001</v>
-      </c>
+    <row r="47" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
       <c r="D47" s="9"/>
-      <c r="E47" s="9">
-        <v>0.20599999999999999</v>
-      </c>
-      <c r="F47" s="9">
-        <v>0.38</v>
-      </c>
-      <c r="G47" s="10">
-        <v>0.98599999999999999</v>
-      </c>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="10"/>
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
       <c r="J47" s="7"/>
@@ -2704,26 +2320,13 @@
       <c r="X47" s="7"/>
       <c r="Y47" s="8"/>
     </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="1">
-        <v>1996</v>
-      </c>
-      <c r="B48" s="9">
-        <v>18368.52</v>
-      </c>
-      <c r="C48" s="9">
-        <v>127.04</v>
-      </c>
+    <row r="48" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
       <c r="D48" s="9"/>
-      <c r="E48" s="9">
-        <v>0.28199999999999997</v>
-      </c>
-      <c r="F48" s="9">
-        <v>0.34499999999999997</v>
-      </c>
-      <c r="G48" s="10">
-        <v>0.96599999999999997</v>
-      </c>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="10"/>
       <c r="H48" s="7"/>
       <c r="I48" s="7"/>
       <c r="J48" s="7"/>
@@ -2743,26 +2346,13 @@
       <c r="X48" s="7"/>
       <c r="Y48" s="8"/>
     </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="1">
-        <v>1997</v>
-      </c>
-      <c r="B49" s="9">
-        <v>24455.99</v>
-      </c>
-      <c r="C49" s="9">
-        <v>130.96299999999999</v>
-      </c>
+    <row r="49" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
       <c r="D49" s="9"/>
-      <c r="E49" s="9">
-        <v>0.26700000000000002</v>
-      </c>
-      <c r="F49" s="9">
-        <v>0.33100000000000002</v>
-      </c>
-      <c r="G49" s="10">
-        <v>0.94199999999999995</v>
-      </c>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="10"/>
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
       <c r="J49" s="7"/>
@@ -2782,26 +2372,13 @@
       <c r="X49" s="7"/>
       <c r="Y49" s="8"/>
     </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A50" s="1">
-        <v>1998</v>
-      </c>
-      <c r="B50" s="9">
-        <v>16861.5</v>
-      </c>
-      <c r="C50" s="9">
-        <v>130.42400000000001</v>
-      </c>
+    <row r="50" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B50" s="9"/>
+      <c r="C50" s="9"/>
       <c r="D50" s="9"/>
-      <c r="E50" s="9">
-        <v>0.22500000000000001</v>
-      </c>
-      <c r="F50" s="9">
-        <v>0.3</v>
-      </c>
-      <c r="G50" s="10">
-        <v>0.92400000000000004</v>
-      </c>
+      <c r="E50" s="9"/>
+      <c r="F50" s="9"/>
+      <c r="G50" s="10"/>
       <c r="H50" s="7"/>
       <c r="I50" s="7"/>
       <c r="J50" s="7"/>
@@ -2821,26 +2398,13 @@
       <c r="X50" s="7"/>
       <c r="Y50" s="8"/>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A51" s="1">
-        <v>1999</v>
-      </c>
-      <c r="B51" s="9">
-        <v>22340.51</v>
-      </c>
-      <c r="C51" s="9">
-        <v>121.89700000000001</v>
-      </c>
+    <row r="51" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B51" s="9"/>
+      <c r="C51" s="9"/>
       <c r="D51" s="9"/>
-      <c r="E51" s="9">
-        <v>0.251</v>
-      </c>
-      <c r="F51" s="9">
-        <v>0.2</v>
-      </c>
-      <c r="G51" s="10">
-        <v>0.92300000000000004</v>
-      </c>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="10"/>
       <c r="H51" s="7"/>
       <c r="I51" s="7"/>
       <c r="J51" s="7"/>
@@ -2860,26 +2424,13 @@
       <c r="X51" s="7"/>
       <c r="Y51" s="8"/>
     </row>
-    <row r="52" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A52" s="1">
-        <v>2000</v>
-      </c>
-      <c r="B52" s="9">
-        <v>28945.602999999999</v>
-      </c>
-      <c r="C52" s="9">
-        <v>117.292</v>
-      </c>
+    <row r="52" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
       <c r="D52" s="9"/>
-      <c r="E52" s="9">
-        <v>0.29799999999999999</v>
-      </c>
-      <c r="F52" s="9">
-        <v>0.187</v>
-      </c>
-      <c r="G52" s="10">
-        <v>0.92700000000000005</v>
-      </c>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
+      <c r="G52" s="10"/>
       <c r="H52" s="7"/>
       <c r="I52" s="7"/>
       <c r="J52" s="7"/>
@@ -2899,404 +2450,157 @@
       <c r="X52" s="7"/>
       <c r="Y52" s="8"/>
     </row>
-    <row r="53" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A53" s="1">
-        <v>2001</v>
-      </c>
-      <c r="B53" s="11">
-        <v>21181.764999999999</v>
-      </c>
-      <c r="C53" s="11">
-        <v>129.786</v>
-      </c>
+    <row r="53" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B53" s="11"/>
+      <c r="C53" s="11"/>
       <c r="D53" s="11"/>
-      <c r="E53" s="11">
-        <v>0.246</v>
-      </c>
-      <c r="F53" s="11">
-        <v>0.26800000000000002</v>
-      </c>
-      <c r="G53" s="12">
-        <v>0.86199999999999999</v>
-      </c>
-    </row>
-    <row r="54" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="1">
-        <v>2002</v>
-      </c>
-      <c r="B54" s="11">
-        <v>26016.432000000001</v>
-      </c>
-      <c r="C54" s="11">
-        <v>165.142</v>
-      </c>
+      <c r="E53" s="11"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="12"/>
+    </row>
+    <row r="54" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B54" s="11"/>
+      <c r="C54" s="11"/>
       <c r="D54" s="11"/>
-      <c r="E54" s="11">
-        <v>0.22600000000000001</v>
-      </c>
-      <c r="F54" s="11">
-        <v>0.59299999999999997</v>
-      </c>
-      <c r="G54" s="12">
-        <v>0.87</v>
-      </c>
-    </row>
-    <row r="55" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A55" s="1">
-        <v>2003</v>
-      </c>
-      <c r="B55" s="11">
-        <v>33361.798000000003</v>
-      </c>
-      <c r="C55" s="11">
-        <v>160.28800000000001</v>
-      </c>
+      <c r="E54" s="11"/>
+      <c r="F54" s="11"/>
+      <c r="G54" s="12"/>
+    </row>
+    <row r="55" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B55" s="11"/>
+      <c r="C55" s="11"/>
       <c r="D55" s="11"/>
-      <c r="E55" s="11">
-        <v>0.122</v>
-      </c>
-      <c r="F55" s="11">
-        <v>0.65</v>
-      </c>
-      <c r="G55" s="12">
-        <v>0.86599999999999999</v>
-      </c>
-    </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A56" s="1">
-        <v>2004</v>
-      </c>
-      <c r="B56" s="11">
-        <v>40935.357000000004</v>
-      </c>
-      <c r="C56" s="11">
-        <v>161.298</v>
-      </c>
+      <c r="E55" s="11"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="12"/>
+    </row>
+    <row r="56" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B56" s="11"/>
+      <c r="C56" s="11"/>
       <c r="D56" s="11"/>
-      <c r="E56" s="11">
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="F56" s="11">
-        <v>0.60899999999999999</v>
-      </c>
-      <c r="G56" s="12">
-        <v>0.88600000000000001</v>
-      </c>
-    </row>
-    <row r="57" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A57" s="1">
-        <v>2005</v>
-      </c>
-      <c r="B57" s="11">
-        <v>43858.196000000004</v>
-      </c>
-      <c r="C57" s="11">
-        <v>182.59299999999999</v>
-      </c>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="12"/>
+    </row>
+    <row r="57" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
       <c r="D57" s="11"/>
-      <c r="E57" s="11">
-        <v>0.23899999999999999</v>
-      </c>
-      <c r="F57" s="11">
-        <v>0.73199999999999998</v>
-      </c>
-      <c r="G57" s="12">
-        <v>0.91800000000000004</v>
-      </c>
-    </row>
-    <row r="58" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A58" s="1">
-        <v>2006</v>
-      </c>
-      <c r="B58" s="11">
-        <v>40590.555</v>
-      </c>
-      <c r="C58" s="11">
-        <v>185.51</v>
-      </c>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="12"/>
+    </row>
+    <row r="58" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B58" s="11"/>
+      <c r="C58" s="11"/>
       <c r="D58" s="11"/>
-      <c r="E58" s="11">
-        <v>0.19600000000000001</v>
-      </c>
-      <c r="F58" s="11">
-        <v>0.74199999999999999</v>
-      </c>
-      <c r="G58" s="12">
-        <v>0.93799999999999994</v>
-      </c>
-    </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A59" s="1">
-        <v>2007</v>
-      </c>
-      <c r="B59" s="11">
-        <v>38639.050999999999</v>
-      </c>
-      <c r="C59" s="11">
-        <v>167.86099999999999</v>
-      </c>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="12"/>
+    </row>
+    <row r="59" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B59" s="11"/>
+      <c r="C59" s="11"/>
       <c r="D59" s="11"/>
-      <c r="E59" s="11">
-        <v>0.25600000000000001</v>
-      </c>
-      <c r="F59" s="11">
-        <v>0.61399999999999999</v>
-      </c>
-      <c r="G59" s="12">
-        <v>0.93300000000000005</v>
-      </c>
-    </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A60" s="1">
-        <v>2008</v>
-      </c>
-      <c r="B60" s="11">
-        <v>42523.642</v>
-      </c>
-      <c r="C60" s="11">
-        <v>177.22</v>
-      </c>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="12"/>
+    </row>
+    <row r="60" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B60" s="11"/>
+      <c r="C60" s="11"/>
       <c r="D60" s="11"/>
-      <c r="E60" s="11">
-        <v>0.19</v>
-      </c>
-      <c r="F60" s="11">
-        <v>0.70099999999999996</v>
-      </c>
-      <c r="G60" s="12">
-        <v>0.91500000000000004</v>
-      </c>
-    </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A61" s="1">
-        <v>2009</v>
-      </c>
-      <c r="B61" s="11">
-        <v>48428.983999999997</v>
-      </c>
-      <c r="C61" s="11">
-        <v>181.24700000000001</v>
-      </c>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+      <c r="G60" s="12"/>
+    </row>
+    <row r="61" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B61" s="11"/>
+      <c r="C61" s="11"/>
       <c r="D61" s="11"/>
-      <c r="E61" s="11">
-        <v>0.20399999999999999</v>
-      </c>
-      <c r="F61" s="11">
-        <v>0.79</v>
-      </c>
-      <c r="G61" s="12">
-        <v>0.88600000000000001</v>
-      </c>
-    </row>
-    <row r="62" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A62" s="1">
-        <v>2010</v>
-      </c>
-      <c r="B62" s="11">
-        <v>46505.906000000003</v>
-      </c>
-      <c r="C62" s="11">
-        <v>171.405</v>
-      </c>
+      <c r="E61" s="11"/>
+      <c r="F61" s="11"/>
+      <c r="G61" s="12"/>
+    </row>
+    <row r="62" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B62" s="11"/>
+      <c r="C62" s="11"/>
       <c r="D62" s="11"/>
-      <c r="E62" s="11">
-        <v>0.218</v>
-      </c>
-      <c r="F62" s="11">
-        <v>0.71599999999999997</v>
-      </c>
-      <c r="G62" s="12">
-        <v>0.85099999999999998</v>
-      </c>
-    </row>
-    <row r="63" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="1">
-        <v>2011</v>
-      </c>
-      <c r="B63" s="11">
-        <v>48861.785000000003</v>
-      </c>
-      <c r="C63" s="11">
-        <v>189.49100000000001</v>
-      </c>
+      <c r="E62" s="11"/>
+      <c r="F62" s="11"/>
+      <c r="G62" s="12"/>
+    </row>
+    <row r="63" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B63" s="11"/>
+      <c r="C63" s="11"/>
       <c r="D63" s="11"/>
-      <c r="E63" s="11">
-        <v>0.155</v>
-      </c>
-      <c r="F63" s="11">
-        <v>0.83799999999999997</v>
-      </c>
-      <c r="G63" s="12">
-        <v>0.81599999999999995</v>
-      </c>
-    </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A64" s="1">
-        <v>2012</v>
-      </c>
-      <c r="B64" s="11">
-        <v>52250.358999999997</v>
-      </c>
-      <c r="C64" s="11">
-        <v>184.49600000000001</v>
-      </c>
+      <c r="E63" s="11"/>
+      <c r="F63" s="11"/>
+      <c r="G63" s="12"/>
+    </row>
+    <row r="64" spans="2:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="B64" s="11"/>
+      <c r="C64" s="11"/>
       <c r="D64" s="11"/>
-      <c r="E64" s="11">
-        <v>0.2</v>
-      </c>
-      <c r="F64" s="11">
-        <v>0.84499999999999997</v>
-      </c>
-      <c r="G64" s="12">
-        <v>0.77800000000000002</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A65" s="1">
-        <v>2013</v>
-      </c>
-      <c r="B65" s="11">
-        <v>56494.726999999999</v>
-      </c>
-      <c r="C65" s="11">
-        <v>173.03700000000001</v>
-      </c>
+      <c r="E64" s="11"/>
+      <c r="F64" s="11"/>
+      <c r="G64" s="12"/>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="B65" s="11"/>
+      <c r="C65" s="11"/>
       <c r="D65" s="11"/>
-      <c r="E65" s="11">
-        <v>0.22800000000000001</v>
-      </c>
-      <c r="F65" s="11">
-        <v>0.71299999999999997</v>
-      </c>
-      <c r="G65" s="12">
-        <v>0.75800000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A66" s="1">
-        <v>2014</v>
-      </c>
-      <c r="B66" s="11">
-        <v>54756.72</v>
-      </c>
-      <c r="C66" s="11">
-        <v>172.56299999999999</v>
-      </c>
+      <c r="E65" s="11"/>
+      <c r="F65" s="11"/>
+      <c r="G65" s="12"/>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="B66" s="11"/>
+      <c r="C66" s="11"/>
       <c r="D66" s="11"/>
-      <c r="E66" s="11">
-        <v>0.19600000000000001</v>
-      </c>
-      <c r="F66" s="11">
-        <v>0.77700000000000002</v>
-      </c>
-      <c r="G66" s="12">
-        <v>0.70799999999999996</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A67" s="1">
-        <v>2015</v>
-      </c>
-      <c r="B67" s="11">
-        <v>50794.01</v>
-      </c>
-      <c r="C67" s="11">
-        <v>180.40600000000001</v>
-      </c>
+      <c r="E66" s="11"/>
+      <c r="F66" s="11"/>
+      <c r="G66" s="12"/>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="B67" s="11"/>
+      <c r="C67" s="11"/>
       <c r="D67" s="11"/>
-      <c r="E67" s="11">
-        <v>0.19900000000000001</v>
-      </c>
-      <c r="F67" s="11">
-        <v>0.73</v>
-      </c>
-      <c r="G67" s="12">
-        <v>0.67900000000000005</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A68" s="1">
-        <v>2016</v>
-      </c>
-      <c r="B68" s="11">
-        <v>55308.288</v>
-      </c>
-      <c r="C68" s="11">
-        <v>189.18299999999999</v>
-      </c>
+      <c r="E67" s="11"/>
+      <c r="F67" s="11"/>
+      <c r="G67" s="12"/>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="B68" s="11"/>
+      <c r="C68" s="11"/>
       <c r="D68" s="11"/>
-      <c r="E68" s="11">
-        <v>0.22500000000000001</v>
-      </c>
-      <c r="F68" s="11">
-        <v>0.81799999999999995</v>
-      </c>
-      <c r="G68" s="12">
-        <v>0.65400000000000003</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A69" s="1">
-        <v>2017</v>
-      </c>
-      <c r="B69" s="11">
-        <v>57529.906999999999</v>
-      </c>
-      <c r="C69" s="11">
-        <v>181.44900000000001</v>
-      </c>
+      <c r="E68" s="11"/>
+      <c r="F68" s="11"/>
+      <c r="G68" s="12"/>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="B69" s="11"/>
+      <c r="C69" s="11"/>
       <c r="D69" s="11"/>
-      <c r="E69" s="11">
-        <v>0.222</v>
-      </c>
-      <c r="F69" s="11">
-        <v>0.70899999999999996</v>
-      </c>
-      <c r="G69" s="12">
-        <v>0.61</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A70" s="1">
-        <v>2018</v>
-      </c>
-      <c r="B70" s="11">
-        <v>37030.906000000003</v>
-      </c>
-      <c r="C70" s="11">
-        <v>170.81100000000001</v>
-      </c>
+      <c r="E69" s="11"/>
+      <c r="F69" s="11"/>
+      <c r="G69" s="12"/>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="B70" s="11"/>
+      <c r="C70" s="11"/>
       <c r="D70" s="11"/>
-      <c r="E70" s="11">
-        <v>0.23300000000000001</v>
-      </c>
-      <c r="F70" s="11">
-        <v>0.69599999999999995</v>
-      </c>
-      <c r="G70" s="12">
-        <v>0.58299999999999996</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A71" s="1">
-        <v>2019</v>
-      </c>
-      <c r="B71" s="11">
-        <v>43240.186999999998</v>
-      </c>
-      <c r="C71" s="11">
-        <v>177.78800000000001</v>
-      </c>
+      <c r="E70" s="11"/>
+      <c r="F70" s="11"/>
+      <c r="G70" s="12"/>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="B71" s="11"/>
+      <c r="C71" s="11"/>
       <c r="D71" s="11"/>
-      <c r="E71" s="11">
-        <v>0.20399999999999999</v>
-      </c>
-      <c r="F71" s="11">
-        <v>0.77700000000000002</v>
-      </c>
-      <c r="G71" s="12">
-        <v>0.57599999999999996</v>
-      </c>
+      <c r="E71" s="11"/>
+      <c r="F71" s="11"/>
+      <c r="G71" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>